<commit_message>
Triệu: V5 phân tích B2 so với B0 + đề xuất nhánh P
Bản đề xuất nằm tại reports/TRIEU_DE_XUAT_NHANH_P_20261029.md (đã gửi Trí, bàn buổi 03/11).
</commit_message>
<xml_diff>
--- a/reports/audits/TRIEU_TINH_TAY.xlsx
+++ b/reports/audits/TRIEU_TINH_TAY.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diosodumb\Documents\CS331\reports\audits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF942F53-DB66-4DA8-89D3-E128A198853B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9ABEC3-35B7-49F7-9A4C-07B3662E0F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" activeTab="2" xr2:uid="{D94D246F-C79F-41E1-9EFD-53C8DB4BF0A9}"/>
+    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="16220" activeTab="3" xr2:uid="{D94D246F-C79F-41E1-9EFD-53C8DB4BF0A9}"/>
   </bookViews>
   <sheets>
     <sheet name="TRIEU_TINH_TAY" sheetId="1" r:id="rId1"/>
     <sheet name="q05_2" sheetId="2" r:id="rId2"/>
     <sheet name="ca_hong" sheetId="3" r:id="rId3"/>
+    <sheet name="tap_moi" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="137">
   <si>
     <t>query_id</t>
   </si>
@@ -257,6 +258,195 @@
   </si>
   <si>
     <t>Đoán đúng 2/5. Dữ liệu sai định dạng → dừng; lỗi chạy ghi đúng quy ước (error + null) → cho qua, loại khỏi so sánh cả B0 lẫn B2 và báo coverage. File hỏng tạo từ bản sao m4_first5_b0, file gốc không bị sửa.</t>
+  </si>
+  <si>
+    <t>delta</t>
+  </si>
+  <si>
+    <t>compare_B0_B2</t>
+  </si>
+  <si>
+    <t>u01_1</t>
+  </si>
+  <si>
+    <t>u01_2</t>
+  </si>
+  <si>
+    <t>u01_3</t>
+  </si>
+  <si>
+    <t>u02_1</t>
+  </si>
+  <si>
+    <t>u02_2</t>
+  </si>
+  <si>
+    <t>u02_3</t>
+  </si>
+  <si>
+    <t>u03_1</t>
+  </si>
+  <si>
+    <t>u03_2</t>
+  </si>
+  <si>
+    <t>u03_3</t>
+  </si>
+  <si>
+    <t>u04_1</t>
+  </si>
+  <si>
+    <t>u04_2</t>
+  </si>
+  <si>
+    <t>u04_3</t>
+  </si>
+  <si>
+    <t>u05_1</t>
+  </si>
+  <si>
+    <t>u05_2</t>
+  </si>
+  <si>
+    <t>u05_3</t>
+  </si>
+  <si>
+    <t>u06_1</t>
+  </si>
+  <si>
+    <t>u06_2</t>
+  </si>
+  <si>
+    <t>u06_3</t>
+  </si>
+  <si>
+    <t>u07_1</t>
+  </si>
+  <si>
+    <t>u07_2</t>
+  </si>
+  <si>
+    <t>u07_3</t>
+  </si>
+  <si>
+    <t>u08_1</t>
+  </si>
+  <si>
+    <t>u08_2</t>
+  </si>
+  <si>
+    <t>u08_3</t>
+  </si>
+  <si>
+    <t>u09_1</t>
+  </si>
+  <si>
+    <t>u09_2</t>
+  </si>
+  <si>
+    <t>u09_3</t>
+  </si>
+  <si>
+    <t>u10_1</t>
+  </si>
+  <si>
+    <t>u10_2</t>
+  </si>
+  <si>
+    <t>u10_3</t>
+  </si>
+  <si>
+    <t>prompt</t>
+  </si>
+  <si>
+    <t>people</t>
+  </si>
+  <si>
+    <t>dogs</t>
+  </si>
+  <si>
+    <t>sheep</t>
+  </si>
+  <si>
+    <t>cats</t>
+  </si>
+  <si>
+    <t>amplifiers</t>
+  </si>
+  <si>
+    <t>bicycles</t>
+  </si>
+  <si>
+    <t>guitars</t>
+  </si>
+  <si>
+    <t>chairs</t>
+  </si>
+  <si>
+    <t>beach umbrellas</t>
+  </si>
+  <si>
+    <t>forks</t>
+  </si>
+  <si>
+    <t>blackberries</t>
+  </si>
+  <si>
+    <t>cars</t>
+  </si>
+  <si>
+    <t>boats</t>
+  </si>
+  <si>
+    <t>trucks</t>
+  </si>
+  <si>
+    <t>motorbikes</t>
+  </si>
+  <si>
+    <t>presence</t>
+  </si>
+  <si>
+    <t>gt</t>
+  </si>
+  <si>
+    <t>present</t>
+  </si>
+  <si>
+    <t>absent</t>
+  </si>
+  <si>
+    <t>pred_B0</t>
+  </si>
+  <si>
+    <t>pred_B2_original</t>
+  </si>
+  <si>
+    <t>MAE B0 (30 query)</t>
+  </si>
+  <si>
+    <t>MAE B2 (30 query)</t>
+  </si>
+  <si>
+    <t>MAE B0 (chỉ có mặt)</t>
+  </si>
+  <si>
+    <t>MAE B2 (chỉ có mặt)</t>
+  </si>
+  <si>
+    <t>absent, B0 &gt; 0</t>
+  </si>
+  <si>
+    <t>absent, B2 &gt; 0</t>
+  </si>
+  <si>
+    <t>MAE B0 bỏ u10_2</t>
+  </si>
+  <si>
+    <t>MAE B2 bỏ u10_2</t>
+  </si>
+  <si>
+    <t>chỉ</t>
   </si>
 </sst>
 </file>
@@ -1142,7 +1332,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93938754-808F-48EF-A61E-50A290196CEB}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="17.125" customWidth="1"/>
@@ -1154,9 +1344,10 @@
     <col min="7" max="7" width="14.625" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="11.875" customWidth="1"/>
+    <col min="11" max="11" width="16.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1184,8 +1375,14 @@
       <c r="I1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" t="s">
+        <v>74</v>
+      </c>
+      <c r="K1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1218,8 +1415,16 @@
         <f>IF(F2&lt;E2,"improved",IF(F2&gt;E2,"worsened","unchanged"))</f>
         <v>unchanged</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="J2">
+        <f>F2-E2</f>
+        <v>0</v>
+      </c>
+      <c r="K2" t="str">
+        <f>IF(J2&lt;0,"B2 better",IF(J2&gt;0,"B2 worse","same"))</f>
+        <v>same</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1252,8 +1457,16 @@
         <f t="shared" ref="I3:I16" si="4">IF(F3&lt;E3,"improved",IF(F3&gt;E3,"worsened","unchanged"))</f>
         <v>improved</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="J3">
+        <f t="shared" ref="J3:J16" si="5">F3-E3</f>
+        <v>-6</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K16" si="6">IF(J3&lt;0,"B2 better",IF(J3&gt;0,"B2 worse","same"))</f>
+        <v>B2 better</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1286,8 +1499,16 @@
         <f t="shared" si="4"/>
         <v>unchanged</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="J4">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="6"/>
+        <v>same</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1320,8 +1541,16 @@
         <f t="shared" si="4"/>
         <v>worsened</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="J5">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 worse</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1354,8 +1583,16 @@
         <f t="shared" si="4"/>
         <v>unchanged</v>
       </c>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="J6">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="6"/>
+        <v>same</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1388,8 +1625,16 @@
         <f t="shared" si="4"/>
         <v>worsened</v>
       </c>
-    </row>
-    <row r="8" spans="1:9">
+      <c r="J7">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="K7" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 worse</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1422,8 +1667,16 @@
         <f t="shared" si="4"/>
         <v>improved</v>
       </c>
-    </row>
-    <row r="9" spans="1:9">
+      <c r="J8">
+        <f t="shared" si="5"/>
+        <v>-4</v>
+      </c>
+      <c r="K8" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 better</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1456,8 +1709,16 @@
         <f t="shared" si="4"/>
         <v>unchanged</v>
       </c>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="J9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="K9" t="str">
+        <f t="shared" si="6"/>
+        <v>same</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1490,8 +1751,16 @@
         <f t="shared" si="4"/>
         <v>improved</v>
       </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="J10">
+        <f t="shared" si="5"/>
+        <v>-1</v>
+      </c>
+      <c r="K10" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 better</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1524,8 +1793,16 @@
         <f t="shared" si="4"/>
         <v>improved</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
+      <c r="J11">
+        <f t="shared" si="5"/>
+        <v>-1</v>
+      </c>
+      <c r="K11" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 better</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1558,8 +1835,16 @@
         <f t="shared" si="4"/>
         <v>improved</v>
       </c>
-    </row>
-    <row r="13" spans="1:9">
+      <c r="J12">
+        <f t="shared" si="5"/>
+        <v>-11</v>
+      </c>
+      <c r="K12" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 better</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1592,8 +1877,16 @@
         <f t="shared" si="4"/>
         <v>unchanged</v>
       </c>
-    </row>
-    <row r="14" spans="1:9">
+      <c r="J13">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="K13" t="str">
+        <f t="shared" si="6"/>
+        <v>same</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1626,8 +1919,16 @@
         <f t="shared" si="4"/>
         <v>improved</v>
       </c>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="J14">
+        <f t="shared" si="5"/>
+        <v>-5</v>
+      </c>
+      <c r="K14" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 better</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1660,8 +1961,16 @@
         <f t="shared" si="4"/>
         <v>worsened</v>
       </c>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="J15">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="K15" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 worse</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1693,6 +2002,14 @@
       <c r="I16" t="str">
         <f t="shared" si="4"/>
         <v>worsened</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="5"/>
+        <v>58</v>
+      </c>
+      <c r="K16" t="str">
+        <f t="shared" si="6"/>
+        <v>B2 worse</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2168,4 +2485,1228 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2FDACE-9D41-42D0-B50E-DCA0BA62263F}">
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="17.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>14</v>
+      </c>
+      <c r="F2">
+        <v>38</v>
+      </c>
+      <c r="G2">
+        <f>ABS(E2-D2)</f>
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <f>ABS(F2-D2)</f>
+        <v>28</v>
+      </c>
+      <c r="I2">
+        <f>H2-G2</f>
+        <v>24</v>
+      </c>
+      <c r="J2" s="2" t="str">
+        <f>IF(H2&lt;G2,"improved",IF(H2&gt;G2,"worsened","unchanged"))</f>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3">
+        <v>27</v>
+      </c>
+      <c r="E3">
+        <v>32</v>
+      </c>
+      <c r="F3">
+        <v>31</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G31" si="0">ABS(E3-D3)</f>
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H31" si="1">ABS(F3-D3)</f>
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I31" si="2">H3-G3</f>
+        <v>-1</v>
+      </c>
+      <c r="J3" s="2" t="str">
+        <f t="shared" ref="J3:J31" si="3">IF(H3&lt;G3,"improved",IF(H3&gt;G3,"worsened","unchanged"))</f>
+        <v>improved</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>32</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="J4" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>15</v>
+      </c>
+      <c r="F5">
+        <v>20</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="J5" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6">
+        <v>20</v>
+      </c>
+      <c r="E6">
+        <v>18</v>
+      </c>
+      <c r="F6">
+        <v>19</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="2"/>
+        <v>-1</v>
+      </c>
+      <c r="J6" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>improved</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>12</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="J8" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
+      <c r="E12">
+        <v>8</v>
+      </c>
+      <c r="F12">
+        <v>9</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>24</v>
+      </c>
+      <c r="F14">
+        <v>29</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="J14" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D15">
+        <v>24</v>
+      </c>
+      <c r="E15">
+        <v>24</v>
+      </c>
+      <c r="F15">
+        <v>26</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="J15" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" t="s">
+        <v>125</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" t="s">
+        <v>124</v>
+      </c>
+      <c r="D17">
+        <v>23</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+      <c r="F17">
+        <v>49</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="J17" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18">
+        <v>30</v>
+      </c>
+      <c r="E18">
+        <v>31</v>
+      </c>
+      <c r="F18">
+        <v>31</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" t="s">
+        <v>125</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20">
+        <v>6</v>
+      </c>
+      <c r="E20">
+        <v>7</v>
+      </c>
+      <c r="F20">
+        <v>21</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="J20" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D21">
+        <v>22</v>
+      </c>
+      <c r="E21">
+        <v>22</v>
+      </c>
+      <c r="F21">
+        <v>22</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>21</v>
+      </c>
+      <c r="F22">
+        <v>24</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="J22" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23">
+        <v>7</v>
+      </c>
+      <c r="E23">
+        <v>16</v>
+      </c>
+      <c r="F23">
+        <v>20</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="J23" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" t="s">
+        <v>124</v>
+      </c>
+      <c r="D24">
+        <v>14</v>
+      </c>
+      <c r="E24">
+        <v>13</v>
+      </c>
+      <c r="F24">
+        <v>13</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J25" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" t="s">
+        <v>124</v>
+      </c>
+      <c r="D26">
+        <v>30</v>
+      </c>
+      <c r="E26">
+        <v>29</v>
+      </c>
+      <c r="F26">
+        <v>28</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="J26" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" t="s">
+        <v>119</v>
+      </c>
+      <c r="C27" t="s">
+        <v>124</v>
+      </c>
+      <c r="D27">
+        <v>8</v>
+      </c>
+      <c r="E27">
+        <v>8</v>
+      </c>
+      <c r="F27">
+        <v>8</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" t="s">
+        <v>125</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>unchanged</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29">
+        <v>27</v>
+      </c>
+      <c r="E29">
+        <v>54</v>
+      </c>
+      <c r="F29">
+        <v>72</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="J29" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" t="s">
+        <v>104</v>
+      </c>
+      <c r="B30" t="s">
+        <v>121</v>
+      </c>
+      <c r="C30" t="s">
+        <v>124</v>
+      </c>
+      <c r="D30">
+        <v>17</v>
+      </c>
+      <c r="E30">
+        <v>33</v>
+      </c>
+      <c r="F30">
+        <v>80</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="2"/>
+        <v>47</v>
+      </c>
+      <c r="J30" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" t="s">
+        <v>112</v>
+      </c>
+      <c r="C31" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>48</v>
+      </c>
+      <c r="F31">
+        <v>75</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="J31" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>worsened</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B34">
+        <f>AVERAGE(G2:G31)</f>
+        <v>6.7666666666666666</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>129</v>
+      </c>
+      <c r="B35">
+        <f>AVERAGE(H2:H31)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36">
+        <f>AVERAGEIF(C2:C31,"present",G2:G31)</f>
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>131</v>
+      </c>
+      <c r="B37">
+        <f>AVERAGEIF(C2:C31,"present",H2:H31)</f>
+        <v>12.95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>28</v>
+      </c>
+      <c r="B38">
+        <f>COUNTIF(J2:J31,"improved")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>29</v>
+      </c>
+      <c r="B39">
+        <f>COUNTIF(J2:J31,"worsened")</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40">
+        <f>COUNTIF(J2:J31,"unchanged")</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41">
+        <f>COUNTIFS(C2:C31,"absent",E2:E31,"&gt;0")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42">
+        <f>COUNTIFS(C2:C31,"absent",F2:F31,"&gt;0")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44">
+        <f>(SUM(G2:G31)-G30)/29</f>
+        <v>6.4482758620689653</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>135</v>
+      </c>
+      <c r="B45" t="s">
+        <v>136</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>